<commit_message>
done, not fully tested
</commit_message>
<xml_diff>
--- a/data/export-final.xlsx
+++ b/data/export-final.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,6 +26,7 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font/>
   </fonts>
   <fills count="2">
     <fill>
@@ -47,8 +48,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment textRotation="90"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -414,168 +418,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Acinetobacter baumannii NCTC 13301 (OXA-23 + OXA-51-like)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Candida albicans ATCC 90028 = CCM 8161</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Enterococcus faecalis ATCC 29212 = CCM 4224</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Enterococcus faecium 419/ANA </t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Escherichia coli 20574/C</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Escherichia coli ATCC 25922 = CCM 3954</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Escherichia coli CE5556 </t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Escherichia coli NCTC 13846 = CCM 8874 (COL R)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Klebsiella pneumoniae NCTC 13438 (KPC-3)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Klebsiella pneumoniae NCTC 13443 (NDM-1)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Proteus mirabilis 16585/B</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Pseudomonas aeruginosa ATCC 27853 = CCM 3955</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Pseudomonas aeruginosa R</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Staphylococcus aureus 4591</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Staphylococcus aureus ATCC 29213 = CCM 4223</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Staphylococcus epidermidis CCM 7221</t>
         </is>
       </c>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
+      <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
+      <c r="AA1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>I76DR_1037P1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>128</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>128</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -584,7 +608,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>&gt;128</t>
+          <t>I76NS_231P1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -658,6 +682,11 @@
         </is>
       </c>
       <c r="P3" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>&gt;128</t>
         </is>
@@ -666,7 +695,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>&gt;128</t>
+          <t>I76NS_233P1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -740,6 +769,11 @@
         </is>
       </c>
       <c r="P4" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>&gt;128</t>
         </is>
@@ -748,7 +782,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>&gt;128</t>
+          <t>I76NS_235P1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -822,6 +856,11 @@
         </is>
       </c>
       <c r="P5" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>&gt;128</t>
         </is>
@@ -830,7 +869,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>&gt;128</t>
+          <t>I76NS_240P1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -840,14 +879,14 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
           <t>64</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>&gt;128</t>
@@ -855,24 +894,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>64</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>128</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>&gt;128</t>
@@ -895,15 +934,20 @@
       </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>32</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>16</t>
         </is>
@@ -912,15 +956,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
+          <t>I76NS_241P1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>&gt;128</t>
@@ -982,6 +1026,11 @@
         </is>
       </c>
       <c r="P7" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>&gt;128</t>
         </is>
@@ -998,168 +1047,188 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:AA7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Acinetobacter baumannii NCTC 13301 (OXA-23 + OXA-51-like)</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Candida albicans ATCC 90028 = CCM 8161</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Enterococcus faecalis ATCC 29212 = CCM 4224</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Enterococcus faecium 419/ANA </t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Escherichia coli 20574/C</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Escherichia coli ATCC 25922 = CCM 3954</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Escherichia coli CE5556 </t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Escherichia coli NCTC 13846 = CCM 8874 (COL R)</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Klebsiella pneumoniae NCTC 13438 (KPC-3)</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Klebsiella pneumoniae NCTC 13443 (NDM-1)</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Proteus mirabilis 16585/B</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Pseudomonas aeruginosa ATCC 27853 = CCM 3955</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Pseudomonas aeruginosa R</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Staphylococcus aureus 4591</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Staphylococcus aureus ATCC 29213 = CCM 4223</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Staphylococcus epidermidis CCM 7221</t>
         </is>
       </c>
+      <c r="R1" s="1" t="n"/>
+      <c r="S1" s="1" t="n"/>
+      <c r="T1" s="1" t="n"/>
+      <c r="U1" s="1" t="n"/>
+      <c r="V1" s="1" t="n"/>
+      <c r="W1" s="1" t="n"/>
+      <c r="X1" s="1" t="n"/>
+      <c r="Y1" s="1" t="n"/>
+      <c r="Z1" s="1" t="n"/>
+      <c r="AA1" s="1" t="n"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>I76DR_1037P1</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>128</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="D2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>32</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
           <t>32</t>
         </is>
       </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="L2" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
+      <c r="O2" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="O2" t="inlineStr">
+      <c r="P2" t="inlineStr">
         <is>
           <t>0.5</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
+      <c r="Q2" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -1168,7 +1237,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>&gt;128</t>
+          <t>I76NS_231P1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1242,6 +1311,11 @@
         </is>
       </c>
       <c r="P3" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>&gt;128</t>
         </is>
@@ -1250,7 +1324,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>&gt;128</t>
+          <t>I76NS_233P1</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1324,6 +1398,11 @@
         </is>
       </c>
       <c r="P4" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
         <is>
           <t>&gt;128</t>
         </is>
@@ -1332,7 +1411,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>&gt;128</t>
+          <t>I76NS_235P1</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -1406,6 +1485,11 @@
         </is>
       </c>
       <c r="P5" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
         <is>
           <t>&gt;128</t>
         </is>
@@ -1414,24 +1498,24 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>&gt;128</t>
+          <t>I76NS_240P1</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
           <t>128</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>64</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>&gt;128</t>
@@ -1439,24 +1523,24 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>64</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="H6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
           <t>64</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="J6" t="inlineStr">
         <is>
           <t>&gt;128</t>
@@ -1469,25 +1553,30 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
           <t>128</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
       <c r="N6" t="inlineStr">
         <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
           <t>16</t>
         </is>
       </c>
-      <c r="O6" t="inlineStr">
+      <c r="P6" t="inlineStr">
         <is>
           <t>16</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
+      <c r="Q6" t="inlineStr">
         <is>
           <t>16</t>
         </is>
@@ -1496,15 +1585,15 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>&gt;128</t>
-        </is>
-      </c>
+          <t>I76NS_241P1</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
           <t>&gt;128</t>
@@ -1566,6 +1655,11 @@
         </is>
       </c>
       <c r="P7" t="inlineStr">
+        <is>
+          <t>&gt;128</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
         <is>
           <t>&gt;128</t>
         </is>

</xml_diff>